<commit_message>
Add validation early stopping and heuristic link baselines
</commit_message>
<xml_diff>
--- a/results/graph_results.xlsx
+++ b/results/graph_results.xlsx
@@ -515,13 +515,13 @@
         </is>
       </c>
       <c r="J2" t="n">
-        <v>40.8</v>
+        <v>70.53</v>
       </c>
       <c r="K2" t="n">
         <v>386</v>
       </c>
       <c r="L2" t="n">
-        <v>357.4</v>
+        <v>368.34</v>
       </c>
     </row>
     <row r="3">

</xml_diff>

<commit_message>
Add graph cross-validation metrics aggregation
</commit_message>
<xml_diff>
--- a/results/graph_results.xlsx
+++ b/results/graph_results.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L17"/>
+  <dimension ref="A1:O17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -477,6 +477,21 @@
           <t>Memory_MB</t>
         </is>
       </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>Precision</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>Recall</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -523,6 +538,9 @@
       <c r="L2" t="n">
         <v>368.34</v>
       </c>
+      <c r="M2" t="inlineStr"/>
+      <c r="N2" t="inlineStr"/>
+      <c r="O2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -569,6 +587,9 @@
       <c r="L3" t="n">
         <v>379.39</v>
       </c>
+      <c r="M3" t="inlineStr"/>
+      <c r="N3" t="inlineStr"/>
+      <c r="O3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -615,6 +636,9 @@
       <c r="L4" t="n">
         <v>359.32</v>
       </c>
+      <c r="M4" t="inlineStr"/>
+      <c r="N4" t="inlineStr"/>
+      <c r="O4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -653,13 +677,22 @@
         </is>
       </c>
       <c r="J5" t="n">
-        <v>38.58</v>
+        <v>95.19</v>
       </c>
       <c r="K5" t="n">
         <v>1442</v>
       </c>
       <c r="L5" t="n">
-        <v>359.74</v>
+        <v>359.78</v>
+      </c>
+      <c r="M5" t="n">
+        <v>0.8004</v>
+      </c>
+      <c r="N5" t="n">
+        <v>0.7539</v>
+      </c>
+      <c r="O5" t="n">
+        <v>0.7347</v>
       </c>
     </row>
     <row r="6">
@@ -707,6 +740,9 @@
       <c r="L6" t="n">
         <v>403.61</v>
       </c>
+      <c r="M6" t="inlineStr"/>
+      <c r="N6" t="inlineStr"/>
+      <c r="O6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -753,6 +789,9 @@
       <c r="L7" t="n">
         <v>465.53</v>
       </c>
+      <c r="M7" t="inlineStr"/>
+      <c r="N7" t="inlineStr"/>
+      <c r="O7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -799,6 +838,9 @@
       <c r="L8" t="n">
         <v>395.89</v>
       </c>
+      <c r="M8" t="inlineStr"/>
+      <c r="N8" t="inlineStr"/>
+      <c r="O8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -845,6 +887,9 @@
       <c r="L9" t="n">
         <v>400.85</v>
       </c>
+      <c r="M9" t="inlineStr"/>
+      <c r="N9" t="inlineStr"/>
+      <c r="O9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -891,6 +936,9 @@
       <c r="L10" t="n">
         <v>375.13</v>
       </c>
+      <c r="M10" t="inlineStr"/>
+      <c r="N10" t="inlineStr"/>
+      <c r="O10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -937,6 +985,9 @@
       <c r="L11" t="n">
         <v>426.58</v>
       </c>
+      <c r="M11" t="inlineStr"/>
+      <c r="N11" t="inlineStr"/>
+      <c r="O11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -983,6 +1034,9 @@
       <c r="L12" t="n">
         <v>382.38</v>
       </c>
+      <c r="M12" t="inlineStr"/>
+      <c r="N12" t="inlineStr"/>
+      <c r="O12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1029,6 +1083,9 @@
       <c r="L13" t="n">
         <v>379.52</v>
       </c>
+      <c r="M13" t="inlineStr"/>
+      <c r="N13" t="inlineStr"/>
+      <c r="O13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1075,6 +1132,9 @@
       <c r="L14" t="n">
         <v>482.47</v>
       </c>
+      <c r="M14" t="inlineStr"/>
+      <c r="N14" t="inlineStr"/>
+      <c r="O14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1121,6 +1181,9 @@
       <c r="L15" t="n">
         <v>501.7</v>
       </c>
+      <c r="M15" t="inlineStr"/>
+      <c r="N15" t="inlineStr"/>
+      <c r="O15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1167,6 +1230,9 @@
       <c r="L16" t="n">
         <v>480.57</v>
       </c>
+      <c r="M16" t="inlineStr"/>
+      <c r="N16" t="inlineStr"/>
+      <c r="O16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1213,6 +1279,9 @@
       <c r="L17" t="n">
         <v>479.72</v>
       </c>
+      <c r="M17" t="inlineStr"/>
+      <c r="N17" t="inlineStr"/>
+      <c r="O17" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Complete benchmarking improvements and evaluation fixes
</commit_message>
<xml_diff>
--- a/results/graph_results.xlsx
+++ b/results/graph_results.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O17"/>
+  <dimension ref="A1:R17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -492,6 +492,21 @@
           <t>F1</t>
         </is>
       </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>Accuracy_Mean</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>Accuracy_Std</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>ROC_AUC</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -530,17 +545,32 @@
         </is>
       </c>
       <c r="J2" t="n">
-        <v>70.53</v>
+        <v>64.95</v>
       </c>
       <c r="K2" t="n">
-        <v>386</v>
+        <v>1442</v>
       </c>
       <c r="L2" t="n">
-        <v>368.34</v>
-      </c>
-      <c r="M2" t="inlineStr"/>
-      <c r="N2" t="inlineStr"/>
-      <c r="O2" t="inlineStr"/>
+        <v>367.05</v>
+      </c>
+      <c r="M2" t="n">
+        <v>0.7074</v>
+      </c>
+      <c r="N2" t="n">
+        <v>0.64</v>
+      </c>
+      <c r="O2" t="n">
+        <v>0.6413</v>
+      </c>
+      <c r="P2" t="n">
+        <v>0.7126</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>0.0801</v>
+      </c>
+      <c r="R2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -590,6 +620,9 @@
       <c r="M3" t="inlineStr"/>
       <c r="N3" t="inlineStr"/>
       <c r="O3" t="inlineStr"/>
+      <c r="P3" t="inlineStr"/>
+      <c r="Q3" t="inlineStr"/>
+      <c r="R3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -639,6 +672,9 @@
       <c r="M4" t="inlineStr"/>
       <c r="N4" t="inlineStr"/>
       <c r="O4" t="inlineStr"/>
+      <c r="P4" t="inlineStr"/>
+      <c r="Q4" t="inlineStr"/>
+      <c r="R4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -677,13 +713,13 @@
         </is>
       </c>
       <c r="J5" t="n">
-        <v>95.19</v>
+        <v>44.31</v>
       </c>
       <c r="K5" t="n">
         <v>1442</v>
       </c>
       <c r="L5" t="n">
-        <v>359.78</v>
+        <v>366.82</v>
       </c>
       <c r="M5" t="n">
         <v>0.8004</v>
@@ -693,6 +729,15 @@
       </c>
       <c r="O5" t="n">
         <v>0.7347</v>
+      </c>
+      <c r="P5" t="n">
+        <v>0.7719</v>
+      </c>
+      <c r="Q5" t="n">
+        <v>0.1001</v>
+      </c>
+      <c r="R5" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -743,6 +788,9 @@
       <c r="M6" t="inlineStr"/>
       <c r="N6" t="inlineStr"/>
       <c r="O6" t="inlineStr"/>
+      <c r="P6" t="inlineStr"/>
+      <c r="Q6" t="inlineStr"/>
+      <c r="R6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -792,6 +840,9 @@
       <c r="M7" t="inlineStr"/>
       <c r="N7" t="inlineStr"/>
       <c r="O7" t="inlineStr"/>
+      <c r="P7" t="inlineStr"/>
+      <c r="Q7" t="inlineStr"/>
+      <c r="R7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -841,6 +892,9 @@
       <c r="M8" t="inlineStr"/>
       <c r="N8" t="inlineStr"/>
       <c r="O8" t="inlineStr"/>
+      <c r="P8" t="inlineStr"/>
+      <c r="Q8" t="inlineStr"/>
+      <c r="R8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -890,6 +944,9 @@
       <c r="M9" t="inlineStr"/>
       <c r="N9" t="inlineStr"/>
       <c r="O9" t="inlineStr"/>
+      <c r="P9" t="inlineStr"/>
+      <c r="Q9" t="inlineStr"/>
+      <c r="R9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -939,6 +996,9 @@
       <c r="M10" t="inlineStr"/>
       <c r="N10" t="inlineStr"/>
       <c r="O10" t="inlineStr"/>
+      <c r="P10" t="inlineStr"/>
+      <c r="Q10" t="inlineStr"/>
+      <c r="R10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -988,6 +1048,9 @@
       <c r="M11" t="inlineStr"/>
       <c r="N11" t="inlineStr"/>
       <c r="O11" t="inlineStr"/>
+      <c r="P11" t="inlineStr"/>
+      <c r="Q11" t="inlineStr"/>
+      <c r="R11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1037,6 +1100,9 @@
       <c r="M12" t="inlineStr"/>
       <c r="N12" t="inlineStr"/>
       <c r="O12" t="inlineStr"/>
+      <c r="P12" t="inlineStr"/>
+      <c r="Q12" t="inlineStr"/>
+      <c r="R12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1086,6 +1152,9 @@
       <c r="M13" t="inlineStr"/>
       <c r="N13" t="inlineStr"/>
       <c r="O13" t="inlineStr"/>
+      <c r="P13" t="inlineStr"/>
+      <c r="Q13" t="inlineStr"/>
+      <c r="R13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1135,6 +1204,9 @@
       <c r="M14" t="inlineStr"/>
       <c r="N14" t="inlineStr"/>
       <c r="O14" t="inlineStr"/>
+      <c r="P14" t="inlineStr"/>
+      <c r="Q14" t="inlineStr"/>
+      <c r="R14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1184,6 +1256,9 @@
       <c r="M15" t="inlineStr"/>
       <c r="N15" t="inlineStr"/>
       <c r="O15" t="inlineStr"/>
+      <c r="P15" t="inlineStr"/>
+      <c r="Q15" t="inlineStr"/>
+      <c r="R15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1233,6 +1308,9 @@
       <c r="M16" t="inlineStr"/>
       <c r="N16" t="inlineStr"/>
       <c r="O16" t="inlineStr"/>
+      <c r="P16" t="inlineStr"/>
+      <c r="Q16" t="inlineStr"/>
+      <c r="R16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1282,6 +1360,9 @@
       <c r="M17" t="inlineStr"/>
       <c r="N17" t="inlineStr"/>
       <c r="O17" t="inlineStr"/>
+      <c r="P17" t="inlineStr"/>
+      <c r="Q17" t="inlineStr"/>
+      <c r="R17" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Final benchmarking corrections and evaluation updates
</commit_message>
<xml_diff>
--- a/results/graph_results.xlsx
+++ b/results/graph_results.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R17"/>
+  <dimension ref="A1:Q17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -459,52 +459,47 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>Accuracy</t>
+          <t>Accuracy_Mean</t>
         </is>
       </c>
       <c r="J1" t="inlineStr">
         <is>
+          <t>Accuracy_Std</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>Precision</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>Recall</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>ROC_AUC</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
           <t>Training_Time</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>Parameters</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>Memory_MB</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>Precision</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>Recall</t>
-        </is>
-      </c>
-      <c r="O1" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
-      <c r="P1" t="inlineStr">
-        <is>
-          <t>Accuracy_Mean</t>
-        </is>
-      </c>
-      <c r="Q1" t="inlineStr">
-        <is>
-          <t>Accuracy_Std</t>
-        </is>
-      </c>
-      <c r="R1" t="inlineStr">
-        <is>
-          <t>ROC_AUC</t>
         </is>
       </c>
     </row>
@@ -539,37 +534,32 @@
       <c r="H2" t="n">
         <v>200</v>
       </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>0.7389 ± 0.0975</t>
-        </is>
+      <c r="I2" t="n">
+        <v>0.7126</v>
       </c>
       <c r="J2" t="n">
-        <v>64.95</v>
+        <v>0.0801</v>
       </c>
       <c r="K2" t="n">
+        <v>0.7074</v>
+      </c>
+      <c r="L2" t="n">
+        <v>0.64</v>
+      </c>
+      <c r="M2" t="n">
+        <v>0.6413</v>
+      </c>
+      <c r="N2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O2" t="n">
+        <v>54.94</v>
+      </c>
+      <c r="P2" t="n">
         <v>1442</v>
       </c>
-      <c r="L2" t="n">
-        <v>367.05</v>
-      </c>
-      <c r="M2" t="n">
-        <v>0.7074</v>
-      </c>
-      <c r="N2" t="n">
-        <v>0.64</v>
-      </c>
-      <c r="O2" t="n">
-        <v>0.6413</v>
-      </c>
-      <c r="P2" t="n">
-        <v>0.7126</v>
-      </c>
       <c r="Q2" t="n">
-        <v>0.0801</v>
-      </c>
-      <c r="R2" t="n">
-        <v>0</v>
+        <v>361.19</v>
       </c>
     </row>
     <row r="3">
@@ -603,26 +593,33 @@
       <c r="H3" t="n">
         <v>200</v>
       </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>0.7442 ± 0.0958</t>
-        </is>
+      <c r="I3" t="n">
+        <v>0.7442</v>
       </c>
       <c r="J3" t="n">
-        <v>75.40000000000001</v>
+        <v>0.0958</v>
       </c>
       <c r="K3" t="n">
+        <v>0.713</v>
+      </c>
+      <c r="L3" t="n">
+        <v>0.6755</v>
+      </c>
+      <c r="M3" t="n">
+        <v>0.6603</v>
+      </c>
+      <c r="N3" t="n">
+        <v>0</v>
+      </c>
+      <c r="O3" t="n">
+        <v>75.78</v>
+      </c>
+      <c r="P3" t="n">
         <v>3590</v>
       </c>
-      <c r="L3" t="n">
-        <v>379.39</v>
-      </c>
-      <c r="M3" t="inlineStr"/>
-      <c r="N3" t="inlineStr"/>
-      <c r="O3" t="inlineStr"/>
-      <c r="P3" t="inlineStr"/>
-      <c r="Q3" t="inlineStr"/>
-      <c r="R3" t="inlineStr"/>
+      <c r="Q3" t="n">
+        <v>379.25</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -655,26 +652,33 @@
       <c r="H4" t="n">
         <v>200</v>
       </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>0.7602 ± 0.0839</t>
-        </is>
+      <c r="I4" t="n">
+        <v>0.7602</v>
       </c>
       <c r="J4" t="n">
-        <v>37.45</v>
+        <v>0.0839</v>
       </c>
       <c r="K4" t="n">
+        <v>0.7622</v>
+      </c>
+      <c r="L4" t="n">
+        <v>0.7097</v>
+      </c>
+      <c r="M4" t="n">
+        <v>0.707</v>
+      </c>
+      <c r="N4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O4" t="n">
+        <v>37.05</v>
+      </c>
+      <c r="P4" t="n">
         <v>674</v>
       </c>
-      <c r="L4" t="n">
-        <v>359.32</v>
-      </c>
-      <c r="M4" t="inlineStr"/>
-      <c r="N4" t="inlineStr"/>
-      <c r="O4" t="inlineStr"/>
-      <c r="P4" t="inlineStr"/>
-      <c r="Q4" t="inlineStr"/>
-      <c r="R4" t="inlineStr"/>
+      <c r="Q4" t="n">
+        <v>360.05</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -707,37 +711,32 @@
       <c r="H5" t="n">
         <v>200</v>
       </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>0.7719 ± 0.1001</t>
-        </is>
+      <c r="I5" t="n">
+        <v>0.7719</v>
       </c>
       <c r="J5" t="n">
-        <v>44.31</v>
+        <v>0.1001</v>
       </c>
       <c r="K5" t="n">
+        <v>0.8004</v>
+      </c>
+      <c r="L5" t="n">
+        <v>0.7539</v>
+      </c>
+      <c r="M5" t="n">
+        <v>0.7347</v>
+      </c>
+      <c r="N5" t="n">
+        <v>0</v>
+      </c>
+      <c r="O5" t="n">
+        <v>38.24</v>
+      </c>
+      <c r="P5" t="n">
         <v>1442</v>
       </c>
-      <c r="L5" t="n">
-        <v>366.82</v>
-      </c>
-      <c r="M5" t="n">
-        <v>0.8004</v>
-      </c>
-      <c r="N5" t="n">
-        <v>0.7539</v>
-      </c>
-      <c r="O5" t="n">
-        <v>0.7347</v>
-      </c>
-      <c r="P5" t="n">
-        <v>0.7719</v>
-      </c>
       <c r="Q5" t="n">
-        <v>0.1001</v>
-      </c>
-      <c r="R5" t="n">
-        <v>0</v>
+        <v>359.85</v>
       </c>
     </row>
     <row r="6">
@@ -771,26 +770,33 @@
       <c r="H6" t="n">
         <v>200</v>
       </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>0.6623 ± 0.0433</t>
-        </is>
+      <c r="I6" t="n">
+        <v>0.6811</v>
       </c>
       <c r="J6" t="n">
-        <v>280.77</v>
+        <v>0.06619999999999999</v>
       </c>
       <c r="K6" t="n">
-        <v>258</v>
+        <v>0.6841</v>
       </c>
       <c r="L6" t="n">
-        <v>403.61</v>
-      </c>
-      <c r="M6" t="inlineStr"/>
-      <c r="N6" t="inlineStr"/>
-      <c r="O6" t="inlineStr"/>
-      <c r="P6" t="inlineStr"/>
-      <c r="Q6" t="inlineStr"/>
-      <c r="R6" t="inlineStr"/>
+        <v>0.6476</v>
+      </c>
+      <c r="M6" t="n">
+        <v>0.6414</v>
+      </c>
+      <c r="N6" t="n">
+        <v>0</v>
+      </c>
+      <c r="O6" t="n">
+        <v>442.15</v>
+      </c>
+      <c r="P6" t="n">
+        <v>1314</v>
+      </c>
+      <c r="Q6" t="n">
+        <v>409.09</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -823,26 +829,33 @@
       <c r="H7" t="n">
         <v>200</v>
       </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>0.6793 ± 0.0508</t>
-        </is>
+      <c r="I7" t="n">
+        <v>0.6793</v>
       </c>
       <c r="J7" t="n">
-        <v>674.4299999999999</v>
+        <v>0.0508</v>
       </c>
       <c r="K7" t="n">
+        <v>0.6714</v>
+      </c>
+      <c r="L7" t="n">
+        <v>0.6657999999999999</v>
+      </c>
+      <c r="M7" t="n">
+        <v>0.6621</v>
+      </c>
+      <c r="N7" t="n">
+        <v>0</v>
+      </c>
+      <c r="O7" t="n">
+        <v>680.65</v>
+      </c>
+      <c r="P7" t="n">
         <v>2566</v>
       </c>
-      <c r="L7" t="n">
-        <v>465.53</v>
-      </c>
-      <c r="M7" t="inlineStr"/>
-      <c r="N7" t="inlineStr"/>
-      <c r="O7" t="inlineStr"/>
-      <c r="P7" t="inlineStr"/>
-      <c r="Q7" t="inlineStr"/>
-      <c r="R7" t="inlineStr"/>
+      <c r="Q7" t="n">
+        <v>465.77</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -875,26 +888,33 @@
       <c r="H8" t="n">
         <v>200</v>
       </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>0.6766 ± 0.0606</t>
-        </is>
+      <c r="I8" t="n">
+        <v>0.6766</v>
       </c>
       <c r="J8" t="n">
-        <v>248.43</v>
+        <v>0.0606</v>
       </c>
       <c r="K8" t="n">
+        <v>0.6723</v>
+      </c>
+      <c r="L8" t="n">
+        <v>0.641</v>
+      </c>
+      <c r="M8" t="n">
+        <v>0.6419</v>
+      </c>
+      <c r="N8" t="n">
+        <v>0</v>
+      </c>
+      <c r="O8" t="n">
+        <v>247.66</v>
+      </c>
+      <c r="P8" t="n">
         <v>418</v>
       </c>
-      <c r="L8" t="n">
-        <v>395.89</v>
-      </c>
-      <c r="M8" t="inlineStr"/>
-      <c r="N8" t="inlineStr"/>
-      <c r="O8" t="inlineStr"/>
-      <c r="P8" t="inlineStr"/>
-      <c r="Q8" t="inlineStr"/>
-      <c r="R8" t="inlineStr"/>
+      <c r="Q8" t="n">
+        <v>397.34</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -927,26 +947,33 @@
       <c r="H9" t="n">
         <v>200</v>
       </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>0.6829 ± 0.0396</t>
-        </is>
+      <c r="I9" t="n">
+        <v>0.6829</v>
       </c>
       <c r="J9" t="n">
-        <v>331.38</v>
+        <v>0.0396</v>
       </c>
       <c r="K9" t="n">
+        <v>0.6771</v>
+      </c>
+      <c r="L9" t="n">
+        <v>0.6657999999999999</v>
+      </c>
+      <c r="M9" t="n">
+        <v>0.6629</v>
+      </c>
+      <c r="N9" t="n">
+        <v>0</v>
+      </c>
+      <c r="O9" t="n">
+        <v>327.42</v>
+      </c>
+      <c r="P9" t="n">
         <v>1314</v>
       </c>
-      <c r="L9" t="n">
-        <v>400.85</v>
-      </c>
-      <c r="M9" t="inlineStr"/>
-      <c r="N9" t="inlineStr"/>
-      <c r="O9" t="inlineStr"/>
-      <c r="P9" t="inlineStr"/>
-      <c r="Q9" t="inlineStr"/>
-      <c r="R9" t="inlineStr"/>
+      <c r="Q9" t="n">
+        <v>400.48</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -979,26 +1006,33 @@
       <c r="H10" t="n">
         <v>200</v>
       </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>0.3033 ± 0.0332</t>
-        </is>
+      <c r="I10" t="n">
+        <v>0.3017</v>
       </c>
       <c r="J10" t="n">
-        <v>147.29</v>
+        <v>0.0376</v>
       </c>
       <c r="K10" t="n">
-        <v>390</v>
+        <v>0.2957</v>
       </c>
       <c r="L10" t="n">
-        <v>375.13</v>
-      </c>
-      <c r="M10" t="inlineStr"/>
-      <c r="N10" t="inlineStr"/>
-      <c r="O10" t="inlineStr"/>
-      <c r="P10" t="inlineStr"/>
-      <c r="Q10" t="inlineStr"/>
-      <c r="R10" t="inlineStr"/>
+        <v>0.2978</v>
+      </c>
+      <c r="M10" t="n">
+        <v>0.2631</v>
+      </c>
+      <c r="N10" t="n">
+        <v>0.6474</v>
+      </c>
+      <c r="O10" t="n">
+        <v>187.27</v>
+      </c>
+      <c r="P10" t="n">
+        <v>1446</v>
+      </c>
+      <c r="Q10" t="n">
+        <v>382.64</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1031,26 +1065,33 @@
       <c r="H11" t="n">
         <v>200</v>
       </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>0.2667 ± 0.0453</t>
-        </is>
+      <c r="I11" t="n">
+        <v>0.2667</v>
       </c>
       <c r="J11" t="n">
-        <v>341.86</v>
+        <v>0.0453</v>
       </c>
       <c r="K11" t="n">
+        <v>0.2419</v>
+      </c>
+      <c r="L11" t="n">
+        <v>0.272</v>
+      </c>
+      <c r="M11" t="n">
+        <v>0.2268</v>
+      </c>
+      <c r="N11" t="n">
+        <v>0.6254999999999999</v>
+      </c>
+      <c r="O11" t="n">
+        <v>338.44</v>
+      </c>
+      <c r="P11" t="n">
         <v>3602</v>
       </c>
-      <c r="L11" t="n">
-        <v>426.58</v>
-      </c>
-      <c r="M11" t="inlineStr"/>
-      <c r="N11" t="inlineStr"/>
-      <c r="O11" t="inlineStr"/>
-      <c r="P11" t="inlineStr"/>
-      <c r="Q11" t="inlineStr"/>
-      <c r="R11" t="inlineStr"/>
+      <c r="Q11" t="n">
+        <v>427.09</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1083,26 +1124,33 @@
       <c r="H12" t="n">
         <v>200</v>
       </c>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>0.3133 ± 0.0371</t>
-        </is>
+      <c r="I12" t="n">
+        <v>0.3133</v>
       </c>
       <c r="J12" t="n">
-        <v>126.34</v>
+        <v>0.0371</v>
       </c>
       <c r="K12" t="n">
+        <v>0.3022</v>
+      </c>
+      <c r="L12" t="n">
+        <v>0.3172</v>
+      </c>
+      <c r="M12" t="n">
+        <v>0.2871</v>
+      </c>
+      <c r="N12" t="n">
+        <v>0.6546999999999999</v>
+      </c>
+      <c r="O12" t="n">
+        <v>125.88</v>
+      </c>
+      <c r="P12" t="n">
         <v>678</v>
       </c>
-      <c r="L12" t="n">
-        <v>382.38</v>
-      </c>
-      <c r="M12" t="inlineStr"/>
-      <c r="N12" t="inlineStr"/>
-      <c r="O12" t="inlineStr"/>
-      <c r="P12" t="inlineStr"/>
-      <c r="Q12" t="inlineStr"/>
-      <c r="R12" t="inlineStr"/>
+      <c r="Q12" t="n">
+        <v>383.79</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1135,26 +1183,33 @@
       <c r="H13" t="n">
         <v>200</v>
       </c>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>0.3133 ± 0.0452</t>
-        </is>
+      <c r="I13" t="n">
+        <v>0.3133</v>
       </c>
       <c r="J13" t="n">
-        <v>135.06</v>
+        <v>0.0452</v>
       </c>
       <c r="K13" t="n">
+        <v>0.3205</v>
+      </c>
+      <c r="L13" t="n">
+        <v>0.3161</v>
+      </c>
+      <c r="M13" t="n">
+        <v>0.2836</v>
+      </c>
+      <c r="N13" t="n">
+        <v>0.6689000000000001</v>
+      </c>
+      <c r="O13" t="n">
+        <v>134.89</v>
+      </c>
+      <c r="P13" t="n">
         <v>1446</v>
       </c>
-      <c r="L13" t="n">
-        <v>379.52</v>
-      </c>
-      <c r="M13" t="inlineStr"/>
-      <c r="N13" t="inlineStr"/>
-      <c r="O13" t="inlineStr"/>
-      <c r="P13" t="inlineStr"/>
-      <c r="Q13" t="inlineStr"/>
-      <c r="R13" t="inlineStr"/>
+      <c r="Q13" t="n">
+        <v>380.44</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1187,26 +1242,33 @@
       <c r="H14" t="n">
         <v>200</v>
       </c>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>0.6423 ± 0.0162</t>
-        </is>
+      <c r="I14" t="n">
+        <v>0.6333</v>
       </c>
       <c r="J14" t="n">
-        <v>1705.97</v>
+        <v>0.0179</v>
       </c>
       <c r="K14" t="n">
-        <v>1346</v>
+        <v>0.6511</v>
       </c>
       <c r="L14" t="n">
-        <v>482.47</v>
-      </c>
-      <c r="M14" t="inlineStr"/>
-      <c r="N14" t="inlineStr"/>
-      <c r="O14" t="inlineStr"/>
-      <c r="P14" t="inlineStr"/>
-      <c r="Q14" t="inlineStr"/>
-      <c r="R14" t="inlineStr"/>
+        <v>0.6324</v>
+      </c>
+      <c r="M14" t="n">
+        <v>0.6202</v>
+      </c>
+      <c r="N14" t="n">
+        <v>0</v>
+      </c>
+      <c r="O14" t="n">
+        <v>2032.45</v>
+      </c>
+      <c r="P14" t="n">
+        <v>2402</v>
+      </c>
+      <c r="Q14" t="n">
+        <v>484.59</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1239,26 +1301,33 @@
       <c r="H15" t="n">
         <v>200</v>
       </c>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>0.6078 ± 0.0458</t>
-        </is>
+      <c r="I15" t="n">
+        <v>0.6078</v>
       </c>
       <c r="J15" t="n">
-        <v>3512.28</v>
+        <v>0.0458</v>
       </c>
       <c r="K15" t="n">
+        <v>0.6498</v>
+      </c>
+      <c r="L15" t="n">
+        <v>0.6094000000000001</v>
+      </c>
+      <c r="M15" t="n">
+        <v>0.574</v>
+      </c>
+      <c r="N15" t="n">
+        <v>0</v>
+      </c>
+      <c r="O15" t="n">
+        <v>2936.95</v>
+      </c>
+      <c r="P15" t="n">
         <v>11270</v>
       </c>
-      <c r="L15" t="n">
-        <v>501.7</v>
-      </c>
-      <c r="M15" t="inlineStr"/>
-      <c r="N15" t="inlineStr"/>
-      <c r="O15" t="inlineStr"/>
-      <c r="P15" t="inlineStr"/>
-      <c r="Q15" t="inlineStr"/>
-      <c r="R15" t="inlineStr"/>
+      <c r="Q15" t="n">
+        <v>470.4</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1291,26 +1360,33 @@
       <c r="H16" t="n">
         <v>200</v>
       </c>
-      <c r="I16" t="inlineStr">
-        <is>
-          <t>0.6421 ± 0.0254</t>
-        </is>
+      <c r="I16" t="n">
+        <v>0.6421</v>
       </c>
       <c r="J16" t="n">
-        <v>2958.02</v>
+        <v>0.0254</v>
       </c>
       <c r="K16" t="n">
+        <v>0.6569</v>
+      </c>
+      <c r="L16" t="n">
+        <v>0.6447000000000001</v>
+      </c>
+      <c r="M16" t="n">
+        <v>0.6346000000000001</v>
+      </c>
+      <c r="N16" t="n">
+        <v>0</v>
+      </c>
+      <c r="O16" t="n">
+        <v>1240.12</v>
+      </c>
+      <c r="P16" t="n">
         <v>2594</v>
       </c>
-      <c r="L16" t="n">
-        <v>480.57</v>
-      </c>
-      <c r="M16" t="inlineStr"/>
-      <c r="N16" t="inlineStr"/>
-      <c r="O16" t="inlineStr"/>
-      <c r="P16" t="inlineStr"/>
-      <c r="Q16" t="inlineStr"/>
-      <c r="R16" t="inlineStr"/>
+      <c r="Q16" t="n">
+        <v>482.97</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1343,26 +1419,33 @@
       <c r="H17" t="n">
         <v>200</v>
       </c>
-      <c r="I17" t="inlineStr">
-        <is>
-          <t>0.6888 ± 0.0158</t>
-        </is>
+      <c r="I17" t="n">
+        <v>0.6888</v>
       </c>
       <c r="J17" t="n">
-        <v>2534.12</v>
+        <v>0.0158</v>
       </c>
       <c r="K17" t="n">
+        <v>0.6952</v>
+      </c>
+      <c r="L17" t="n">
+        <v>0.6878</v>
+      </c>
+      <c r="M17" t="n">
+        <v>0.6851</v>
+      </c>
+      <c r="N17" t="n">
+        <v>0</v>
+      </c>
+      <c r="O17" t="n">
+        <v>1971.94</v>
+      </c>
+      <c r="P17" t="n">
         <v>2402</v>
       </c>
-      <c r="L17" t="n">
-        <v>479.72</v>
-      </c>
-      <c r="M17" t="inlineStr"/>
-      <c r="N17" t="inlineStr"/>
-      <c r="O17" t="inlineStr"/>
-      <c r="P17" t="inlineStr"/>
-      <c r="Q17" t="inlineStr"/>
-      <c r="R17" t="inlineStr"/>
+      <c r="Q17" t="n">
+        <v>481.18</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add graph validation split and improve graph benchmarking
</commit_message>
<xml_diff>
--- a/results/graph_results.xlsx
+++ b/results/graph_results.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q17"/>
+  <dimension ref="A1:Q18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1447,6 +1447,65 @@
         <v>481.18</v>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>graph</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>gcn</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>MUTAG</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>32</v>
+      </c>
+      <c r="E18" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="F18" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="G18" t="n">
+        <v>0.0005</v>
+      </c>
+      <c r="H18" t="n">
+        <v>200</v>
+      </c>
+      <c r="I18" t="n">
+        <v>0.7175</v>
+      </c>
+      <c r="J18" t="n">
+        <v>0.1106</v>
+      </c>
+      <c r="K18" t="n">
+        <v>0.6977</v>
+      </c>
+      <c r="L18" t="n">
+        <v>0.6803</v>
+      </c>
+      <c r="M18" t="n">
+        <v>0.6567</v>
+      </c>
+      <c r="N18" t="n">
+        <v>0.7419</v>
+      </c>
+      <c r="O18" t="n">
+        <v>52.67</v>
+      </c>
+      <c r="P18" t="n">
+        <v>1506</v>
+      </c>
+      <c r="Q18" t="n">
+        <v>362.16</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Complete graph validation and benchmarking fixes
</commit_message>
<xml_diff>
--- a/results/graph_results.xlsx
+++ b/results/graph_results.xlsx
@@ -1479,31 +1479,31 @@
         <v>200</v>
       </c>
       <c r="I18" t="n">
-        <v>0.7175</v>
+        <v>0.7237</v>
       </c>
       <c r="J18" t="n">
-        <v>0.1106</v>
+        <v>0.0833</v>
       </c>
       <c r="K18" t="n">
-        <v>0.6977</v>
+        <v>0.7282999999999999</v>
       </c>
       <c r="L18" t="n">
-        <v>0.6803</v>
+        <v>0.6526</v>
       </c>
       <c r="M18" t="n">
-        <v>0.6567</v>
+        <v>0.6497000000000001</v>
       </c>
       <c r="N18" t="n">
-        <v>0.7419</v>
+        <v>0.7998</v>
       </c>
       <c r="O18" t="n">
-        <v>52.67</v>
+        <v>14.47</v>
       </c>
       <c r="P18" t="n">
         <v>1506</v>
       </c>
       <c r="Q18" t="n">
-        <v>362.16</v>
+        <v>361.8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>